<commit_message>
Remove duplicated camiseta (base64) + regenerate Excel: 50 prendas, guía de cuidados, dropdowns N/O/P
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mi_Guardarropa.xlsx
+++ b/Mi_Guardarropa.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Referencia Zonas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Referencia Armonías" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Guía cuidados" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,35 +27,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -65,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -73,178 +48,10 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001A1A1A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="005B8DB8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8E8E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006B2737"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CC2200"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B8D4E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4820A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00AAEE22"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001A2744"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00222222"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDDDDD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00111111"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F0E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF69B4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0022BB55"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E05070"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002255CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="003A5F7A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="008B6914"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B8A882"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006B5A3A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CC3300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00404040"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4E6F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F5E3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCF3CF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8DAEF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDEBD0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001A1A2E"/>
-        <bgColor rgb="001A1A2E"/>
-      </patternFill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -252,146 +59,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -757,116 +433,116 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="35" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
     <col width="6" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="40" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="40" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nombre de la prenda</t>
         </is>
       </c>
-      <c r="C1" s="40" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Zona del cuerpo</t>
         </is>
       </c>
-      <c r="D1" s="40" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E1" s="40" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Subtipo / Largo</t>
         </is>
       </c>
-      <c r="F1" s="40" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Color principal (HEX)</t>
         </is>
       </c>
-      <c r="G1" s="40" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Color secundario (HEX)</t>
         </is>
       </c>
-      <c r="H1" s="40" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Patrón</t>
         </is>
       </c>
-      <c r="I1" s="40" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="J1" s="40" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
       </c>
-      <c r="K1" s="40" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Formalidad</t>
         </is>
       </c>
-      <c r="L1" s="40" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Temporada</t>
         </is>
       </c>
-      <c r="M1" s="40" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="N1" s="40" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Lavado</t>
         </is>
       </c>
-      <c r="O1" s="40" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Secado</t>
         </is>
       </c>
-      <c r="P1" s="40" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Plancha</t>
         </is>
       </c>
-      <c r="Q1" s="40" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Foto</t>
         </is>
       </c>
-      <c r="R1" s="40" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Capa</t>
         </is>
@@ -931,9 +607,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>images/DER85906_1_enlarged.jpg.png</t>
+          <t>images/DER85906_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -990,9 +669,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>images/EMP64361_1_enlarged.jpg.png</t>
+          <t>images/EMP64361_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -1049,9 +731,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>images/ISA250149_3_enlarged.jpg.png</t>
+          <t>images/ISA250149_3_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R4" t="n">
@@ -1113,9 +798,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>images/PERGO20003_1_enlarged.jpg.png</t>
+          <t>images/PERGO20003_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -1172,9 +860,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>images/W12198031_1_enlarged.jpg.png</t>
+          <t>images/W12198031_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -1235,9 +926,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>images/WAVIS64206_1_enlarged.jpg.png</t>
+          <t>images/WAVIS64206_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R7" t="n">
@@ -1298,9 +992,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>images/WDANP20612_1_enlarged.jpg.png</t>
+          <t>images/WDANP20612_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R8" t="n">
@@ -1361,9 +1058,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>images/WIR197626_1_enlarged.jpg.png</t>
+          <t>images/WIR197626_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R9" t="n">
@@ -1420,9 +1120,12 @@
           <t>Primavera/Otoño</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>images/WKS33582_1_enlarged.jpg.png</t>
+          <t>images/WKS33582_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R10" t="n">
@@ -1479,9 +1182,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>images/WKULE31528_1_enlarged.jpg.png</t>
+          <t>images/WKULE31528_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R11" t="n">
@@ -1542,9 +1248,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>images/WL3198924_1_enlarged.jpg.png</t>
+          <t>images/WL3198924_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R12" t="n">
@@ -1605,9 +1314,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>images/WL3200557_1_enlarged.jpg.png</t>
+          <t>images/WL3200557_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R13" t="n">
@@ -1678,9 +1390,12 @@
           <t>Cuello V</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>images/WLCST30215_1_enlarged.jpg.png</t>
+          <t>images/WLCST30215_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R14" t="n">
@@ -1741,9 +1456,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>images/WMCVB25014_1_enlarged.jpg.png</t>
+          <t>images/WMCVB25014_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R15" t="n">
@@ -1809,9 +1527,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>images/WMCVB26435_1_enlarged.jpg.png</t>
+          <t>images/WMCVB26435_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R16" t="n">
@@ -1877,9 +1598,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>images/WNBHD21274_1_enlarged.jpg.png</t>
+          <t>images/WNBHD21274_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R17" t="n">
@@ -1945,9 +1669,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>images/WNOAH23704_1_enlarged.jpg.png</t>
+          <t>images/WNOAH23704_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R18" t="n">
@@ -2013,9 +1740,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>images/WNOAH23949_1_enlarged.jpg.png</t>
+          <t>images/WNOAH23949_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R19" t="n">
@@ -2076,9 +1806,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>images/WPAAI28443_1_enlarged.jpg.png</t>
+          <t>images/WPAAI28443_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R20" t="n">
@@ -2144,9 +1877,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>images/WPRLN128720_1_enlarged.jpg.png</t>
+          <t>images/WPRLN128720_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R21" t="n">
@@ -2217,9 +1953,12 @@
           <t>Ribete verde cuello</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>images/WPRLN134630_1_enlarged.jpg.png</t>
+          <t>images/WPRLN134630_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R22" t="n">
@@ -2276,9 +2015,12 @@
           <t>Primavera/Otoño</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>images/WPRPS21146_1_enlarged.jpg.png</t>
+          <t>images/WPRPS21146_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R23" t="n">
@@ -2335,9 +2077,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>images/WSEEZ20023_1_enlarged.jpg.png</t>
+          <t>images/WSEEZ20023_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R24" t="n">
@@ -2399,9 +2144,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>images/WSTAM21988_1_enlarged.jpg.png</t>
+          <t>images/WSTAM21988_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R25" t="n">
@@ -2472,9 +2220,12 @@
           <t>Cordones azul cielo</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>images/WU2222977_1_enlarged.jpg.png</t>
+          <t>images/WU2222977_1_enlarged.jpg.webp</t>
         </is>
       </c>
       <c r="R26" t="n">
@@ -2531,9 +2282,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>images/IMG_0623 2.png</t>
+          <t>images/IMG_0623_2.webp</t>
         </is>
       </c>
       <c r="R27" t="n">
@@ -2594,9 +2348,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>images/IMG_0624 2.png</t>
+          <t>images/IMG_0624_2.webp</t>
         </is>
       </c>
       <c r="R28" t="n">
@@ -2653,9 +2410,12 @@
           <t>Verano</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>images/IMG_0625 2.png</t>
+          <t>images/IMG_0625_2.webp</t>
         </is>
       </c>
       <c r="R29" t="n">
@@ -2721,9 +2481,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>images/IMG_0626.png</t>
+          <t>images/IMG_0626.webp</t>
         </is>
       </c>
       <c r="R30" t="n">
@@ -2784,9 +2547,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>images/IMG_0627.png</t>
+          <t>images/IMG_0627.webp</t>
         </is>
       </c>
       <c r="R31" t="n">
@@ -2857,9 +2623,12 @@
           <t>Lana</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>images/IMG_0628.png</t>
+          <t>images/IMG_0628.webp</t>
         </is>
       </c>
       <c r="R32" t="n">
@@ -2920,9 +2689,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>images/IMG_0629.png</t>
+          <t>images/IMG_0629.webp</t>
         </is>
       </c>
       <c r="R33" t="n">
@@ -2983,9 +2755,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>images/IMG_0630.png</t>
+          <t>images/IMG_0630.webp</t>
         </is>
       </c>
       <c r="R34" t="n">
@@ -3047,9 +2822,12 @@
           <t>3 botones metálicos</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>images/IMG_0631.png</t>
+          <t>images/IMG_0631.webp</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -3106,9 +2884,12 @@
           <t>Primavera/Otoño</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>images/IMG_0632.png</t>
+          <t>images/IMG_0632.webp</t>
         </is>
       </c>
       <c r="R36" t="n">
@@ -3175,9 +2956,12 @@
           <t>Hair-on-hide</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>images/IMG_0633.png</t>
+          <t>images/IMG_0633.webp</t>
         </is>
       </c>
       <c r="R37" t="n">
@@ -3238,9 +3022,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>images/IMG_0634.png</t>
+          <t>images/IMG_0634.webp</t>
         </is>
       </c>
       <c r="R38" t="n">
@@ -3302,9 +3089,12 @@
           <t>Distressed</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>images/IMG_0635.png</t>
+          <t>images/IMG_0635.webp</t>
         </is>
       </c>
       <c r="R39" t="n">
@@ -3375,9 +3165,12 @@
           <t>Logo A rojo Alabama</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>images/IMG_0636.png</t>
+          <t>images/IMG_0636.webp</t>
         </is>
       </c>
       <c r="R40" t="n">
@@ -3434,9 +3227,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>images/IMG_0637.png</t>
+          <t>images/IMG_0637.webp</t>
         </is>
       </c>
       <c r="R41" t="n">
@@ -3493,9 +3289,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>images/IMG_0638.png</t>
+          <t>images/IMG_0638.webp</t>
         </is>
       </c>
       <c r="R42" t="n">
@@ -3556,9 +3355,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>images/IMG_0639.png</t>
+          <t>images/IMG_0639.webp</t>
         </is>
       </c>
       <c r="R43" t="n">
@@ -3620,9 +3422,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>images/IMG_0640.png</t>
+          <t>images/IMG_0640.webp</t>
         </is>
       </c>
       <c r="R44" t="n">
@@ -3679,9 +3484,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>images/IMG_0641.png</t>
+          <t>images/IMG_0641.webp</t>
         </is>
       </c>
       <c r="R45" t="n">
@@ -3742,9 +3550,12 @@
           <t>Primavera/Verano</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>images/IMG_0642.png</t>
+          <t>images/IMG_0642.webp</t>
         </is>
       </c>
       <c r="R46" t="n">
@@ -3810,9 +3621,12 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>images/IMG_0643.png</t>
+          <t>images/IMG_0643.webp</t>
         </is>
       </c>
       <c r="R47" t="n">
@@ -3869,9 +3683,12 @@
           <t>Otoño/Invierno</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>images/IMG_0644.png</t>
+          <t>images/IMG_0644.webp</t>
         </is>
       </c>
       <c r="R48" t="n">
@@ -3937,9 +3754,12 @@
           <t>Invierno</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>images/IMG_0645.png</t>
+          <t>images/IMG_0645.webp</t>
         </is>
       </c>
       <c r="R49" t="n">
@@ -3996,16 +3816,96 @@
           <t>Todo</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>images/IMG_0646.png</t>
+          <t>images/IMG_0646.webp</t>
         </is>
       </c>
       <c r="R50" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1782716656758</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Camiseta amarilla/negro</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>superior</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Camiseta</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>#f0c048</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Zara</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>casual</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>images/user_1782716644816.webp</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+    </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="N2:N51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"W30,W40,W60,Mano,NoLavar"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Secadora,Tender,NoSecadora"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Baja,Media,Alta,NoPlancha"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4016,343 +3916,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
-        <is>
-          <t>REFERENCIA: Zonas del cuerpo y tipos de prenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="B2" s="31" t="inlineStr">
-        <is>
-          <t>Capas máx.</t>
-        </is>
-      </c>
-      <c r="C2" s="31" t="inlineStr">
-        <is>
-          <t>Tipos de prenda permitidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
-        <is>
-          <t>Cabeza</t>
-        </is>
-      </c>
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>1 capa</t>
-        </is>
-      </c>
-      <c r="C3" s="32" t="inlineStr">
-        <is>
-          <t>Gorra, Sombrero, Beanie, Bucket hat, Visera</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>Cara</t>
-        </is>
-      </c>
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>1 capa</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t>Lentes de sol, Lentes ópticos</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
-        <is>
-          <t>Cuello</t>
-        </is>
-      </c>
-      <c r="B5" s="34" t="inlineStr">
-        <is>
-          <t>2 capas</t>
-        </is>
-      </c>
-      <c r="C5" s="34" t="inlineStr">
-        <is>
-          <t>Bufanda, Paliacate, Pañuelo, Cadena, Collar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
-        <is>
-          <t>Torso</t>
-        </is>
-      </c>
-      <c r="B6" s="35" t="inlineStr">
-        <is>
-          <t>4-5 capas</t>
-        </is>
-      </c>
-      <c r="C6" s="35" t="inlineStr">
-        <is>
-          <t>Camiseta, Camisa, Polo, Tank top, Sudadera, Suéter, Blazer, Chamarra, Abrigo, Chaqueta, Cardigan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
-        <is>
-          <t>Muñeca</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="inlineStr">
-        <is>
-          <t>1 capa</t>
-        </is>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>Reloj, Pulsera, Esclava</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="37" t="inlineStr">
-        <is>
-          <t>Cintura</t>
-        </is>
-      </c>
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>1 capa</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>Cinturón</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
-        <is>
-          <t>Piernas</t>
-        </is>
-      </c>
-      <c r="B9" s="38" t="inlineStr">
-        <is>
-          <t>1 capa</t>
-        </is>
-      </c>
-      <c r="C9" s="38" t="inlineStr">
-        <is>
-          <t>Jean, Pantalón, Short, Jogger, Pants</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>Pies</t>
-        </is>
-      </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>2 capas</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>Calceta (opcional) + Sneakers, Converse, Bota, Zapato, Sandalia, Mocasín</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
-        <is>
-          <t>REFERENCIA: Armonías de Color (Color Wheel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>Armonía</t>
-        </is>
-      </c>
-      <c r="B2" s="31" t="inlineStr">
-        <is>
-          <t>Ángulo en la rueda</t>
-        </is>
-      </c>
-      <c r="C2" s="31" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
-        <is>
-          <t>Monocromática</t>
-        </is>
-      </c>
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>Mismo matiz (0°)</t>
-        </is>
-      </c>
-      <c r="C3" s="32" t="inlineStr">
-        <is>
-          <t>Un solo color en diferentes luminosidades. Ejemplo: azul claro, azul medio, azul oscuro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>Análoga</t>
-        </is>
-      </c>
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>±30° a ±60°</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t>Colores vecinos en la rueda. Resultado natural y armónico. Ejemplo: rojo, naranja, amarillo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
-        <is>
-          <t>Complementaria</t>
-        </is>
-      </c>
-      <c r="B5" s="35" t="inlineStr">
-        <is>
-          <t>180°</t>
-        </is>
-      </c>
-      <c r="C5" s="35" t="inlineStr">
-        <is>
-          <t>Colores opuestos. Máximo contraste. Ejemplo: rojo vs verde, azul vs naranja.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="34" t="inlineStr">
-        <is>
-          <t>Split-Complementaria</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="inlineStr">
-        <is>
-          <t>150° y 210°</t>
-        </is>
-      </c>
-      <c r="C6" s="34" t="inlineStr">
-        <is>
-          <t>Un color + dos adyacentes a su opuesto. Dinámico pero suavizado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
-        <is>
-          <t>Triádica</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="inlineStr">
-        <is>
-          <t>120° y 240°</t>
-        </is>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>Tres colores equidistantes. Vibrante y balanceado. Ejemplo: rojo, azul, amarillo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="37" t="inlineStr">
-        <is>
-          <t>Cuadrada (Square)</t>
-        </is>
-      </c>
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>90°, 180°, 270°</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>Cuatro colores a 90° cada uno. Rica y compleja.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
-        <is>
-          <t>Tetrádica</t>
-        </is>
-      </c>
-      <c r="B9" s="38" t="inlineStr">
-        <is>
-          <t>60° y 120° (rectángulo)</t>
-        </is>
-      </c>
-      <c r="C9" s="38" t="inlineStr">
-        <is>
-          <t>Cuatro colores en rectángulo. La más compleja, requiere un color dominante.</t>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>GUÍA DE VALORES — escribir/elegir EXACTAMENTE como aparece en "Valor exacto"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Columna</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Valor exacto</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lavado (N)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lavadora a 30°C — agua fría, ropa delicada o sintética</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lavado (N)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lavadora a 40°C — algodón y ropa de uso diario</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lavado (N)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>W60</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Lavadora a 60°C — blancos resistentes, toallas, sábanas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lavado (N)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mano</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Solo lavado a mano — lana, seda, viscosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lavado (N)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NoLavar</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>No lavar en casa — solo tintorería (cuero, gamuza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Secado (O)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Secadora</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Aguanta secadora</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Secado (O)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Colgar / tender al aire — no meter a secadora</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Secado (O)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NoSecadora</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nunca secadora — secar en plano o colgado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Plancha (P)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Plancha temperatura baja (1 punto) — sintéticos, lana, seda</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Plancha (P)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Plancha temperatura media (2 puntos) — algodón, mezclas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Plancha (P)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Plancha temperatura alta (3 puntos) — lino, algodón grueso</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Plancha (P)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NoPlancha</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>No planchar — cuero, gamuza, nylon, elastano</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>SUGERENCIA POR MATERIAL (misma tabla que usa la app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Lavado</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Secado</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Plancha</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Algodón</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Secadora</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Lino</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lana</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mano</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Seda</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mano</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bambú</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Lyocell / Tencel</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Viscosa</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Mano</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gamuza</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NoLavar</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>NoPlancha</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cuero</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NoLavar</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NoPlancha</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Poliéster</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Secadora</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nylon</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NoPlancha</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Spandex / Elastano</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tender</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>NoPlancha</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>